<commit_message>
Implement Excel embedded image extraction and Categorized Catalog
</commit_message>
<xml_diff>
--- a/data/Catalogo_Inventario_CreaTuSello.xlsx
+++ b/data/Catalogo_Inventario_CreaTuSello.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>Imagen</t>
   </si>
@@ -143,6 +143,36 @@
   </si>
   <si>
     <t>Solo la montura de madera con mango ergonómico sin goma.</t>
+  </si>
+  <si>
+    <t>LAN-CORP-01</t>
+  </si>
+  <si>
+    <t>Lanyard Corporativo Premium</t>
+  </si>
+  <si>
+    <t>Lanyards</t>
+  </si>
+  <si>
+    <t>90x2cm</t>
+  </si>
+  <si>
+    <t>Correa para el cuello con mosquetón metálico, ideal para portar tu sello.</t>
+  </si>
+  <si>
+    <t>ACC-DIJ-MED</t>
+  </si>
+  <si>
+    <t>Dije Médico (Estetoscopio)</t>
+  </si>
+  <si>
+    <t>Accesorios</t>
+  </si>
+  <si>
+    <t>2x2cm</t>
+  </si>
+  <si>
+    <t>Elegante dije plateado para personalizar tu sello, con temática médica.</t>
   </si>
 </sst>
 </file>
@@ -574,6 +604,84 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="1143000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="1143000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -899,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1143,6 +1251,52 @@
         <v>43</v>
       </c>
     </row>
+    <row r="11" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="G11" s="4">
+        <v>300</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="3">
+        <v>2</v>
+      </c>
+      <c r="G12" s="4">
+        <v>150</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Fix customizer image size, and add CSV generation with URLs
</commit_message>
<xml_diff>
--- a/data/Catalogo_Inventario_CreaTuSello.xlsx
+++ b/data/Catalogo_Inventario_CreaTuSello.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="65">
   <si>
     <t>Imagen</t>
   </si>
@@ -37,6 +37,9 @@
     <t>Descripción</t>
   </si>
   <si>
+    <t>URL de Imagen (Para CSV)</t>
+  </si>
+  <si>
     <t>AUTO-01</t>
   </si>
   <si>
@@ -52,6 +55,9 @@
     <t>Sello automático autoentintable ideal para uso continuo y profesional.</t>
   </si>
   <si>
+    <t>https://lh3.googleusercontent.com/aida-public/AB6AXuDGO80G8SQt65AR4wUkYwUltfDs8LoaK32bXFlaJfKyT_FybVmrmvToGmAOZequsS-1f11vX_hKvryQ22HERLz5fn85KAq6YIeRKPj0b2jKIYjManWEE0GVi7Stz0wvlzudRraK1Z8ckuZt2--OmY3XuP5AQLk5mbwV42vk4NukD7Lo0XCbllu24IAHjaOG708LCn0K09vnaHo0oHg5p29HGk5Jyew0Fddc45hsEch8mJ3AqiaOWkWs46GQ1RSLZFrvxrrfImp9jMg</t>
+  </si>
+  <si>
     <t>FECH-01</t>
   </si>
   <si>
@@ -64,6 +70,9 @@
     <t>Sello con bandas de goma para fechas y texto personalizado superior.</t>
   </si>
   <si>
+    <t>https://lh3.googleusercontent.com/aida-public/AB6AXuD9uzK6LWhBjUP--y4ZuRHJh8T7jJvVMzHrgIkZllVmBHZjhJfD2fzEa5arRBtvj1kzNdSnDJdm67pEDxRJQYk0maCpjODRSVoy6mjwrECSo2ki3E_LPMZJBaMcg8RkNVKMh49N9k3Ka4IbPLaRpygvHNLoFB7p6QO9eUHdWmPkGXMjKuNakmBw1lafVn61CnbA675EIjosRncT6CkKs5cQf74SUmFTFb167DF-fR5GyHLfTzCT0dCfr6zCKsxlYbcVywPV-Uas9rI</t>
+  </si>
+  <si>
     <t>TRAD-01</t>
   </si>
   <si>
@@ -76,6 +85,9 @@
     <t>Sello clásico con montura de madera barnizada. Requiere almohadilla externa.</t>
   </si>
   <si>
+    <t>https://lh3.googleusercontent.com/aida-public/AB6AXuC_B8aoEYQ_lMmCdugdqu_trQMnSWjcCfcnHLHGe1nkRvIk0R-gyzi0PQXawGKDBKywNl2mibxMcSzd8KLlcPFOJ5KapWEgI7tMvp6Zcm_XYrmhpvHCZinpIiRQ8hgpCgMiHHeYntEczPvBzP7Rpozff3eWMgfgD6h-h5hMxoMQmdMk2TnYk-Na6bZYifA-de_DQ8aFxV_gkIN_Ynqv24HleJM_t5_6EeCMChvwwFNyc7JpSZSMBZYY1mUoLriVXIx2ZZ5uA1QwfD8</t>
+  </si>
+  <si>
     <t>PORT-01</t>
   </si>
   <si>
@@ -103,6 +115,9 @@
     <t>Almohadilla de recambio con tinta negra para sellos automáticos estándar.</t>
   </si>
   <si>
+    <t>/repuestos/almohadilla_tinta_negra.png</t>
+  </si>
+  <si>
     <t>REP-ALM-02</t>
   </si>
   <si>
@@ -112,6 +127,9 @@
     <t>Almohadilla de doble color ideal para sellos fechadores.</t>
   </si>
   <si>
+    <t>/repuestos/almohadilla_bicolor.png</t>
+  </si>
+  <si>
     <t>REP-GOM-01</t>
   </si>
   <si>
@@ -124,6 +142,9 @@
     <t>Plantilla de goma cortada a láser con texto o logo personalizado para reemplazo.</t>
   </si>
   <si>
+    <t>/repuestos/goma_grabada.png</t>
+  </si>
+  <si>
     <t>REP-TIN-01</t>
   </si>
   <si>
@@ -136,6 +157,9 @@
     <t>Tinta especial para recargar almohadillas de sellos manuales y automáticos.</t>
   </si>
   <si>
+    <t>/repuestos/frasco_tinta_negra.png</t>
+  </si>
+  <si>
     <t>REP-BAS-01</t>
   </si>
   <si>
@@ -145,6 +169,9 @@
     <t>Solo la montura de madera con mango ergonómico sin goma.</t>
   </si>
   <si>
+    <t>/repuestos/base_madera.png</t>
+  </si>
+  <si>
     <t>LAN-CORP-01</t>
   </si>
   <si>
@@ -160,6 +187,9 @@
     <t>Correa para el cuello con mosquetón metálico, ideal para portar tu sello.</t>
   </si>
   <si>
+    <t>/repuestos/lanyard_corporativo.png</t>
+  </si>
+  <si>
     <t>ACC-DIJ-MED</t>
   </si>
   <si>
@@ -173,6 +203,9 @@
   </si>
   <si>
     <t>Elegante dije plateado para personalizar tu sello, con temática médica.</t>
+  </si>
+  <si>
+    <t>/repuestos/dije_medico.png</t>
   </si>
 </sst>
 </file>
@@ -1007,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1016,9 +1049,10 @@
     <col min="4" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1043,19 +1077,22 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="3">
         <v>19.5</v>
@@ -1064,21 +1101,24 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="3" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3" s="3">
         <v>28</v>
@@ -1087,21 +1127,24 @@
         <v>50</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F4" s="3">
         <v>12</v>
@@ -1110,21 +1153,24 @@
         <v>10</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="5" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F5" s="3">
         <v>22</v>
@@ -1133,21 +1179,24 @@
         <v>75</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="6" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F6" s="3">
         <v>4.5</v>
@@ -1156,21 +1205,24 @@
         <v>200</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="7" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3">
         <v>5.5</v>
@@ -1179,21 +1231,24 @@
         <v>150</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="8" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F8" s="3">
         <v>9</v>
@@ -1202,21 +1257,24 @@
         <v>500</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="9" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F9" s="3">
         <v>6</v>
@@ -1225,21 +1283,24 @@
         <v>80</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F10" s="3">
         <v>5</v>
@@ -1248,21 +1309,24 @@
         <v>30</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>43</v>
+        <v>51</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
-    <row r="11" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F11" s="3">
         <v>3.5</v>
@@ -1271,21 +1335,24 @@
         <v>300</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="12" ht="100" customHeight="1" spans="2:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="100" customHeight="1" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="F12" s="3">
         <v>2</v>
@@ -1294,7 +1361,10 @@
         <v>150</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>53</v>
+        <v>63</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>